<commit_message>
almost all od are done
</commit_message>
<xml_diff>
--- a/Mock_College_ERP.xlsx
+++ b/Mock_College_ERP.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,6 +415,9 @@
       <c r="E1" t="str">
         <v>2026-03-01</v>
       </c>
+      <c r="F1" t="str">
+        <v>2026-03-05</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -432,10 +435,33 @@
       <c r="E2" t="str">
         <v>OD</v>
       </c>
+      <c r="F2" t="str">
+        <v>OD</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>7376222AD168</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Nandhinisakthi Srinivas perumal</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v>OD</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>